<commit_message>
chore: update privacy template assets
</commit_message>
<xml_diff>
--- a/assets/Template_Privacy_Nuovo.xlsx
+++ b/assets/Template_Privacy_Nuovo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UdSAgora\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{205FC6C0-641A-4645-9387-7DCCB548C489}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F152978-52AF-4125-A3A8-D060B19AC56C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-600" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <r>
       <t>Blocco     n.</t>
@@ -617,6 +617,9 @@
   </si>
   <si>
     <t>RICHIESTA NUOVA ASSOCIAZIONE - ANNO 2026/2027</t>
+  </si>
+  <si>
+    <t>TELEFONO</t>
   </si>
 </sst>
 </file>
@@ -886,7 +889,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -932,6 +935,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -1401,12 +1408,12 @@
       <c r="A6" s="4"/>
     </row>
     <row r="7" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="21" t="s">
+      <c r="A7" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="21"/>
-      <c r="C7" s="21"/>
-      <c r="D7" s="21"/>
+      <c r="B7" s="22"/>
+      <c r="C7" s="22"/>
+      <c r="D7" s="22"/>
     </row>
     <row r="8" spans="1:4" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4"/>
@@ -1429,9 +1436,9 @@
       <c r="A11" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B11" s="22"/>
-      <c r="C11" s="22"/>
-      <c r="D11" s="22"/>
+      <c r="B11" s="23"/>
+      <c r="C11" s="23"/>
+      <c r="D11" s="23"/>
     </row>
     <row r="12" spans="1:4" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5"/>
@@ -1455,9 +1462,9 @@
       <c r="A15" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B15" s="22"/>
-      <c r="C15" s="22"/>
-      <c r="D15" s="22"/>
+      <c r="B15" s="23"/>
+      <c r="C15" s="23"/>
+      <c r="D15" s="23"/>
     </row>
     <row r="16" spans="1:4" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="5"/>
@@ -1481,8 +1488,8 @@
       <c r="A19" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B19" s="22"/>
-      <c r="C19" s="22"/>
+      <c r="B19" s="23"/>
+      <c r="C19" s="23"/>
       <c r="D19" s="6" t="s">
         <v>2</v>
       </c>
@@ -1496,8 +1503,10 @@
         <v>12</v>
       </c>
       <c r="B21" s="9"/>
-      <c r="C21" s="5"/>
-      <c r="D21" s="11"/>
+      <c r="C21" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D21" s="15"/>
     </row>
     <row r="22" spans="1:5" ht="11.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="5"/>
@@ -1506,57 +1515,57 @@
       <c r="D22" s="11"/>
     </row>
     <row r="23" spans="1:5" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="25" t="s">
+      <c r="A23" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="B23" s="26"/>
-      <c r="C23" s="26"/>
-      <c r="D23" s="26"/>
+      <c r="B23" s="27"/>
+      <c r="C23" s="27"/>
+      <c r="D23" s="27"/>
     </row>
     <row r="24" spans="1:5" ht="258" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="23" t="s">
+      <c r="A24" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="B24" s="24"/>
-      <c r="C24" s="24"/>
-      <c r="D24" s="24"/>
+      <c r="B24" s="25"/>
+      <c r="C24" s="25"/>
+      <c r="D24" s="25"/>
     </row>
     <row r="25" spans="1:5" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="20"/>
-      <c r="B25" s="20"/>
-      <c r="C25" s="20"/>
-      <c r="D25" s="20"/>
+      <c r="A25" s="21"/>
+      <c r="B25" s="21"/>
+      <c r="C25" s="21"/>
+      <c r="D25" s="21"/>
     </row>
     <row r="26" spans="1:5" s="13" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="17" t="s">
+      <c r="A26" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="B26" s="18"/>
-      <c r="C26" s="18"/>
-      <c r="D26" s="19"/>
+      <c r="B26" s="19"/>
+      <c r="C26" s="19"/>
+      <c r="D26" s="20"/>
       <c r="E26" s="12"/>
     </row>
     <row r="27" spans="1:5" ht="8.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="28"/>
-      <c r="B27" s="28"/>
-      <c r="C27" s="28"/>
-      <c r="D27" s="28"/>
+      <c r="A27" s="29"/>
+      <c r="B27" s="29"/>
+      <c r="C27" s="29"/>
+      <c r="D27" s="29"/>
     </row>
     <row r="28" spans="1:5" ht="265.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="27" t="s">
+      <c r="A28" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="B28" s="27"/>
-      <c r="C28" s="27"/>
-      <c r="D28" s="27"/>
+      <c r="B28" s="28"/>
+      <c r="C28" s="28"/>
+      <c r="D28" s="28"/>
     </row>
     <row r="29" spans="1:5" ht="409.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="15" t="s">
+      <c r="A29" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="B29" s="16"/>
-      <c r="C29" s="16"/>
-      <c r="D29" s="16"/>
+      <c r="B29" s="17"/>
+      <c r="C29" s="17"/>
+      <c r="D29" s="17"/>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="8"/>

</xml_diff>